<commit_message>
Feat: kondisi saat ini
</commit_message>
<xml_diff>
--- a/evaluation/PERTANYAAN_DOKUMEN_with_candidate.xlsx
+++ b/evaluation/PERTANYAAN_DOKUMEN_with_candidate.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anak usia 5-14 tahun menderita anemia dengan presentase 26,4%.</t>
+          <t>prevalensi anemia pada perempuan usia ≥15 tahun sebesar 22,7%</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anak usia 15-24 tahun menderita anemia dengan presentase 18,4%.</t>
+          <t>anak usia 5-14 tahun menderita anemia 26,4% dan usia</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anemia merupakan salah satu masalah kesehatan masyarakat di Indonesia yang dapat dialami oleh semua kelompok umur mulai dari balita, remaja, ibu hamil sampai usia lanjut.</t>
+          <t>BUKU SAKU PENCEGAHAN ANEMIA PADA IBU HAMIL DAN REMAJA PUTRI</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sumber utama vitamin A adalah minyak ikan dan hati sapi. Sumber lain adalah hati.</t>
+          <t>Vitamin A: Sumber utama vitamin A adalah minyak ikan dan hati sapi.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sumber utama vitamin E adalah minyak sayur seperti minyak kelapa, minyak kelapa sawit, dan minyak kacang.</t>
+          <t>Vitamin E: Minyak sayur seperti minyak kelapa, minyak kelapa sawit, dan minyak kacang</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Maaf, saya tidak tahu karena informasi tersebut tidak ada di dokumen.</t>
+          <t>BUKU SAKU PENCEGAHAN ANEMIA PADA IBU HAMIL DAN REMAJA PUTRI</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Prevalensi anemia pada usia 5-14 tahun adalah 26,8%.</t>
+          <t>prevalensi anemia pada perempuan usia ≥15 tahun sebesar 22,7%</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Prevalensi anemia pada usia 15-24 tahun adalah 32%.</t>
+          <t>prevalensi anemia pada perempuan usia ≥15 tahun sebesar 22,7%</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Salah satu target prioritas nasional dalam RPJMN 2020-2024 adalah penurunan stunting menjadi 14% pada tahun 2024 melalui implementasi intervensi gizi spesifik maupun intervensi gizi sensitif.</t>
+          <t>putri (Rematri) merupakan salah satu pelayanan gizi</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TTD tidak berbahaya dan aman dikonsumsi secara rutin, namun konsumsi secara terus menerus perlu mendapat perhatian pada sekelompok populasi yang mempunyai penyakit darah seperti thalassemia, hemosiderosis.</t>
+          <t>Namun, konsumsi TTD secara terus menerus perlu</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Prevalensi anemia pada WUS usia 15 tahun ke atas sebesar 22,7%.</t>
+          <t>prevalensi anemia pada perempuan usia ≥15 tahun sebesar 22,7%</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Prevalensi anemia pada ibu hamil sebesar 37,1%.</t>
+          <t>sedangkan prevalensi anemia pada ibu hamil sebesar 37,1%.</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tujuan umum program penanggulangan anemia pada remaja dan wanita usia subur (WUS) adalah menurunkan prevalensi anemia pada remaja dan WUS.</t>
+          <t>anemia pada rematri dan WUS adalah cakupan program anemia pada</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Prevalensi anemia pada remaja (usia 10-19 tahun) sebesar 30%.</t>
+          <t>55 BUKU SAKU PENCEGAHAN ANEMIA PADA IBU HAMIL DAN REMAJA PUTRI Lampiran 4. Contoh menu dalam 1 kali Makan Kemenkes RI 26 BUKU SAKU PENCEGAHAN ANEMIA PADA IBU HAMIL DAN REMAJA PUTRI B.</t>
         </is>
       </c>
     </row>
@@ -776,13 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Risiko penderita anemia ketika menjadi ibu hamil adalah:
-- Pertumbuhan dan perkembangan janin yang tidak optimal
-- Komplikasi kehamilan dan persalinan
-- Kematian ibu dan anak
-- Meningkatnya risiko persalinan
-- Kematian ibu dan bayi
-- Infeksi penyakit.</t>
+          <t>BUKU SAKU PENCEGAHAN ANEMIA PADA IBU HAMIL DAN REMAJA PUTRI</t>
         </is>
       </c>
     </row>

</xml_diff>